<commit_message>
chore: codex checkpoint (session-stop)
Automatic Codex checkpoint at 2026-08-21 20:23:19.

Reason: session-stop.
</commit_message>
<xml_diff>
--- a/outputs/01a02455-4428-7e10-b65c-4328cbb55411/notas_e_frequencias_metodos_III_2026.xlsx
+++ b/outputs/01a02455-4428-7e10-b65c-4328cbb55411/notas_e_frequencias_metodos_III_2026.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lançamento" sheetId="1" r:id="R2c0844bfc32548de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="2" r:id="R5b05f7017d1e4165"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="3" r:id="R08d9dd6fd8854a40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proveniência" sheetId="4" r:id="Rdacaf23e9f514ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lançamento" sheetId="1" r:id="R7f0c3e6df1b446ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="2" r:id="R2f2cc6f7832a46d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras" sheetId="3" r:id="R6f1bfda51b5e4a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proveniência" sheetId="4" r:id="Ref16f0a8790343f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1379,7 +1379,7 @@
       </x:c>
       <x:c r="D31" s="40" t="n">
         <x:f>'Auditoria'!N31</x:f>
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E31" s="42" t="str">
         <x:f>'Auditoria'!O31</x:f>
@@ -2731,7 +2731,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re13fd2925a6f46c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R101a71aef25443d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2985,7 +2985,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N8" s="37" t="n">
-        <x:f>ROUND(IF(Q8="Não",IF(I8="Não",0,50),MAX(IF(K8&gt;=5,75,0),L8-M8)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q8="Não",IF(I8="Não",0,50),MAX(IF(K8&gt;=5,75,0),L8-M8)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O8" s="41" t="str">
@@ -3054,7 +3054,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N9" s="40" t="n">
-        <x:f>ROUND(IF(Q9="Não",IF(I9="Não",0,50),MAX(IF(K9&gt;=5,75,0),L9-M9)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q9="Não",IF(I9="Não",0,50),MAX(IF(K9&gt;=5,75,0),L9-M9)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O9" s="42" t="str">
@@ -3123,7 +3123,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N10" s="40" t="n">
-        <x:f>ROUND(IF(Q10="Não",IF(I10="Não",0,50),MAX(IF(K10&gt;=5,75,0),L10-M10)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q10="Não",IF(I10="Não",0,50),MAX(IF(K10&gt;=5,75,0),L10-M10)),1),0)</x:f>
         <x:v>89</x:v>
       </x:c>
       <x:c r="O10" s="42" t="str">
@@ -3191,7 +3191,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N11" s="40" t="n">
-        <x:f>ROUND(IF(Q11="Não",IF(I11="Não",0,50),MAX(IF(K11&gt;=5,75,0),L11-M11)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q11="Não",IF(I11="Não",0,50),MAX(IF(K11&gt;=5,75,0),L11-M11)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O11" s="42" t="str">
@@ -3260,7 +3260,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N12" s="40" t="n">
-        <x:f>ROUND(IF(Q12="Não",IF(I12="Não",0,50),MAX(IF(K12&gt;=5,75,0),L12-M12)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q12="Não",IF(I12="Não",0,50),MAX(IF(K12&gt;=5,75,0),L12-M12)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O12" s="42" t="str">
@@ -3329,7 +3329,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N13" s="40" t="n">
-        <x:f>ROUND(IF(Q13="Não",IF(I13="Não",0,50),MAX(IF(K13&gt;=5,75,0),L13-M13)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q13="Não",IF(I13="Não",0,50),MAX(IF(K13&gt;=5,75,0),L13-M13)),1),0)</x:f>
         <x:v>89</x:v>
       </x:c>
       <x:c r="O13" s="42" t="str">
@@ -3398,7 +3398,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N14" s="40" t="n">
-        <x:f>ROUND(IF(Q14="Não",IF(I14="Não",0,50),MAX(IF(K14&gt;=5,75,0),L14-M14)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q14="Não",IF(I14="Não",0,50),MAX(IF(K14&gt;=5,75,0),L14-M14)),1),0)</x:f>
         <x:v>89</x:v>
       </x:c>
       <x:c r="O14" s="42" t="str">
@@ -3466,7 +3466,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N15" s="40" t="n">
-        <x:f>ROUND(IF(Q15="Não",IF(I15="Não",0,50),MAX(IF(K15&gt;=5,75,0),L15-M15)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q15="Não",IF(I15="Não",0,50),MAX(IF(K15&gt;=5,75,0),L15-M15)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O15" s="42" t="str">
@@ -3535,7 +3535,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N16" s="40" t="n">
-        <x:f>ROUND(IF(Q16="Não",IF(I16="Não",0,50),MAX(IF(K16&gt;=5,75,0),L16-M16)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q16="Não",IF(I16="Não",0,50),MAX(IF(K16&gt;=5,75,0),L16-M16)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O16" s="42" t="str">
@@ -3604,7 +3604,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N17" s="40" t="n">
-        <x:f>ROUND(IF(Q17="Não",IF(I17="Não",0,50),MAX(IF(K17&gt;=5,75,0),L17-M17)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q17="Não",IF(I17="Não",0,50),MAX(IF(K17&gt;=5,75,0),L17-M17)),1),0)</x:f>
         <x:v>88</x:v>
       </x:c>
       <x:c r="O17" s="42" t="str">
@@ -3673,7 +3673,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N18" s="40" t="n">
-        <x:f>ROUND(IF(Q18="Não",IF(I18="Não",0,50),MAX(IF(K18&gt;=5,75,0),L18-M18)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q18="Não",IF(I18="Não",0,50),MAX(IF(K18&gt;=5,75,0),L18-M18)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O18" s="42" t="str">
@@ -3741,7 +3741,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N19" s="40" t="n">
-        <x:f>ROUND(IF(Q19="Não",IF(I19="Não",0,50),MAX(IF(K19&gt;=5,75,0),L19-M19)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q19="Não",IF(I19="Não",0,50),MAX(IF(K19&gt;=5,75,0),L19-M19)),1),0)</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="O19" s="42" t="str">
@@ -3810,7 +3810,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N20" s="40" t="n">
-        <x:f>ROUND(IF(Q20="Não",IF(I20="Não",0,50),MAX(IF(K20&gt;=5,75,0),L20-M20)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q20="Não",IF(I20="Não",0,50),MAX(IF(K20&gt;=5,75,0),L20-M20)),1),0)</x:f>
         <x:v>79</x:v>
       </x:c>
       <x:c r="O20" s="42" t="str">
@@ -3878,7 +3878,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N21" s="40" t="n">
-        <x:f>ROUND(IF(Q21="Não",IF(I21="Não",0,50),MAX(IF(K21&gt;=5,75,0),L21-M21)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q21="Não",IF(I21="Não",0,50),MAX(IF(K21&gt;=5,75,0),L21-M21)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O21" s="42" t="str">
@@ -3947,7 +3947,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N22" s="40" t="n">
-        <x:f>ROUND(IF(Q22="Não",IF(I22="Não",0,50),MAX(IF(K22&gt;=5,75,0),L22-M22)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q22="Não",IF(I22="Não",0,50),MAX(IF(K22&gt;=5,75,0),L22-M22)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O22" s="42" t="str">
@@ -4016,7 +4016,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N23" s="40" t="n">
-        <x:f>ROUND(IF(Q23="Não",IF(I23="Não",0,50),MAX(IF(K23&gt;=5,75,0),L23-M23)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q23="Não",IF(I23="Não",0,50),MAX(IF(K23&gt;=5,75,0),L23-M23)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O23" s="42" t="str">
@@ -4084,7 +4084,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N24" s="40" t="n">
-        <x:f>ROUND(IF(Q24="Não",IF(I24="Não",0,50),MAX(IF(K24&gt;=5,75,0),L24-M24)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q24="Não",IF(I24="Não",0,50),MAX(IF(K24&gt;=5,75,0),L24-M24)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O24" s="42" t="str">
@@ -4153,7 +4153,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N25" s="40" t="n">
-        <x:f>ROUND(IF(Q25="Não",IF(I25="Não",0,50),MAX(IF(K25&gt;=5,75,0),L25-M25)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q25="Não",IF(I25="Não",0,50),MAX(IF(K25&gt;=5,75,0),L25-M25)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O25" s="42" t="str">
@@ -4222,7 +4222,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N26" s="40" t="n">
-        <x:f>ROUND(IF(Q26="Não",IF(I26="Não",0,50),MAX(IF(K26&gt;=5,75,0),L26-M26)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q26="Não",IF(I26="Não",0,50),MAX(IF(K26&gt;=5,75,0),L26-M26)),1),0)</x:f>
         <x:v>88</x:v>
       </x:c>
       <x:c r="O26" s="42" t="str">
@@ -4291,7 +4291,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N27" s="40" t="n">
-        <x:f>ROUND(IF(Q27="Não",IF(I27="Não",0,50),MAX(IF(K27&gt;=5,75,0),L27-M27)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q27="Não",IF(I27="Não",0,50),MAX(IF(K27&gt;=5,75,0),L27-M27)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O27" s="42" t="str">
@@ -4360,7 +4360,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N28" s="40" t="n">
-        <x:f>ROUND(IF(Q28="Não",IF(I28="Não",0,50),MAX(IF(K28&gt;=5,75,0),L28-M28)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q28="Não",IF(I28="Não",0,50),MAX(IF(K28&gt;=5,75,0),L28-M28)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O28" s="42" t="str">
@@ -4429,7 +4429,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N29" s="40" t="n">
-        <x:f>ROUND(IF(Q29="Não",IF(I29="Não",0,50),MAX(IF(K29&gt;=5,75,0),L29-M29)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q29="Não",IF(I29="Não",0,50),MAX(IF(K29&gt;=5,75,0),L29-M29)),1),0)</x:f>
         <x:v>89</x:v>
       </x:c>
       <x:c r="O29" s="42" t="str">
@@ -4498,7 +4498,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N30" s="40" t="n">
-        <x:f>ROUND(IF(Q30="Não",IF(I30="Não",0,50),MAX(IF(K30&gt;=5,75,0),L30-M30)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q30="Não",IF(I30="Não",0,50),MAX(IF(K30&gt;=5,75,0),L30-M30)),1),0)</x:f>
         <x:v>89</x:v>
       </x:c>
       <x:c r="O30" s="42" t="str">
@@ -4567,8 +4567,8 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N31" s="40" t="n">
-        <x:f>ROUND(IF(Q31="Não",IF(I31="Não",0,50),MAX(IF(K31&gt;=5,75,0),L31-M31)),0)</x:f>
-        <x:v>89</x:v>
+        <x:f>ROUND(ROUND(IF(Q31="Não",IF(I31="Não",0,50),MAX(IF(K31&gt;=5,75,0),L31-M31)),1),0)</x:f>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="O31" s="42" t="str">
         <x:f>IF(AND(K31&gt;=5,N31&gt;=75),"Aprovado","Reprovado")</x:f>
@@ -4636,7 +4636,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N32" s="40" t="n">
-        <x:f>ROUND(IF(Q32="Não",IF(I32="Não",0,50),MAX(IF(K32&gt;=5,75,0),L32-M32)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q32="Não",IF(I32="Não",0,50),MAX(IF(K32&gt;=5,75,0),L32-M32)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O32" s="42" t="str">
@@ -4705,7 +4705,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N33" s="40" t="n">
-        <x:f>ROUND(IF(Q33="Não",IF(I33="Não",0,50),MAX(IF(K33&gt;=5,75,0),L33-M33)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q33="Não",IF(I33="Não",0,50),MAX(IF(K33&gt;=5,75,0),L33-M33)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O33" s="42" t="str">
@@ -4773,7 +4773,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N34" s="40" t="n">
-        <x:f>ROUND(IF(Q34="Não",IF(I34="Não",0,50),MAX(IF(K34&gt;=5,75,0),L34-M34)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q34="Não",IF(I34="Não",0,50),MAX(IF(K34&gt;=5,75,0),L34-M34)),1),0)</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="O34" s="42" t="str">
@@ -4842,7 +4842,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N35" s="40" t="n">
-        <x:f>ROUND(IF(Q35="Não",IF(I35="Não",0,50),MAX(IF(K35&gt;=5,75,0),L35-M35)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q35="Não",IF(I35="Não",0,50),MAX(IF(K35&gt;=5,75,0),L35-M35)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O35" s="42" t="str">
@@ -4911,7 +4911,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N36" s="40" t="n">
-        <x:f>ROUND(IF(Q36="Não",IF(I36="Não",0,50),MAX(IF(K36&gt;=5,75,0),L36-M36)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q36="Não",IF(I36="Não",0,50),MAX(IF(K36&gt;=5,75,0),L36-M36)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O36" s="42" t="str">
@@ -4980,7 +4980,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N37" s="40" t="n">
-        <x:f>ROUND(IF(Q37="Não",IF(I37="Não",0,50),MAX(IF(K37&gt;=5,75,0),L37-M37)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q37="Não",IF(I37="Não",0,50),MAX(IF(K37&gt;=5,75,0),L37-M37)),1),0)</x:f>
         <x:v>89</x:v>
       </x:c>
       <x:c r="O37" s="42" t="str">
@@ -5049,7 +5049,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N38" s="40" t="n">
-        <x:f>ROUND(IF(Q38="Não",IF(I38="Não",0,50),MAX(IF(K38&gt;=5,75,0),L38-M38)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q38="Não",IF(I38="Não",0,50),MAX(IF(K38&gt;=5,75,0),L38-M38)),1),0)</x:f>
         <x:v>88</x:v>
       </x:c>
       <x:c r="O38" s="42" t="str">
@@ -5118,7 +5118,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N39" s="40" t="n">
-        <x:f>ROUND(IF(Q39="Não",IF(I39="Não",0,50),MAX(IF(K39&gt;=5,75,0),L39-M39)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q39="Não",IF(I39="Não",0,50),MAX(IF(K39&gt;=5,75,0),L39-M39)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O39" s="42" t="str">
@@ -5186,7 +5186,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N40" s="40" t="n">
-        <x:f>ROUND(IF(Q40="Não",IF(I40="Não",0,50),MAX(IF(K40&gt;=5,75,0),L40-M40)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q40="Não",IF(I40="Não",0,50),MAX(IF(K40&gt;=5,75,0),L40-M40)),1),0)</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="O40" s="42" t="str">
@@ -5254,7 +5254,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N41" s="40" t="n">
-        <x:f>ROUND(IF(Q41="Não",IF(I41="Não",0,50),MAX(IF(K41&gt;=5,75,0),L41-M41)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q41="Não",IF(I41="Não",0,50),MAX(IF(K41&gt;=5,75,0),L41-M41)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O41" s="42" t="str">
@@ -5322,7 +5322,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N42" s="40" t="n">
-        <x:f>ROUND(IF(Q42="Não",IF(I42="Não",0,50),MAX(IF(K42&gt;=5,75,0),L42-M42)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q42="Não",IF(I42="Não",0,50),MAX(IF(K42&gt;=5,75,0),L42-M42)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O42" s="42" t="str">
@@ -5391,7 +5391,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N43" s="40" t="n">
-        <x:f>ROUND(IF(Q43="Não",IF(I43="Não",0,50),MAX(IF(K43&gt;=5,75,0),L43-M43)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q43="Não",IF(I43="Não",0,50),MAX(IF(K43&gt;=5,75,0),L43-M43)),1),0)</x:f>
         <x:v>79</x:v>
       </x:c>
       <x:c r="O43" s="42" t="str">
@@ -5460,7 +5460,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N44" s="40" t="n">
-        <x:f>ROUND(IF(Q44="Não",IF(I44="Não",0,50),MAX(IF(K44&gt;=5,75,0),L44-M44)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q44="Não",IF(I44="Não",0,50),MAX(IF(K44&gt;=5,75,0),L44-M44)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O44" s="42" t="str">
@@ -5529,7 +5529,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N45" s="40" t="n">
-        <x:f>ROUND(IF(Q45="Não",IF(I45="Não",0,50),MAX(IF(K45&gt;=5,75,0),L45-M45)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q45="Não",IF(I45="Não",0,50),MAX(IF(K45&gt;=5,75,0),L45-M45)),1),0)</x:f>
         <x:v>79</x:v>
       </x:c>
       <x:c r="O45" s="42" t="str">
@@ -5598,7 +5598,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N46" s="40" t="n">
-        <x:f>ROUND(IF(Q46="Não",IF(I46="Não",0,50),MAX(IF(K46&gt;=5,75,0),L46-M46)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q46="Não",IF(I46="Não",0,50),MAX(IF(K46&gt;=5,75,0),L46-M46)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O46" s="42" t="str">
@@ -5667,7 +5667,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N47" s="40" t="n">
-        <x:f>ROUND(IF(Q47="Não",IF(I47="Não",0,50),MAX(IF(K47&gt;=5,75,0),L47-M47)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q47="Não",IF(I47="Não",0,50),MAX(IF(K47&gt;=5,75,0),L47-M47)),1),0)</x:f>
         <x:v>88</x:v>
       </x:c>
       <x:c r="O47" s="42" t="str">
@@ -5736,7 +5736,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N48" s="40" t="n">
-        <x:f>ROUND(IF(Q48="Não",IF(I48="Não",0,50),MAX(IF(K48&gt;=5,75,0),L48-M48)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q48="Não",IF(I48="Não",0,50),MAX(IF(K48&gt;=5,75,0),L48-M48)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O48" s="42" t="str">
@@ -5805,7 +5805,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N49" s="40" t="n">
-        <x:f>ROUND(IF(Q49="Não",IF(I49="Não",0,50),MAX(IF(K49&gt;=5,75,0),L49-M49)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q49="Não",IF(I49="Não",0,50),MAX(IF(K49&gt;=5,75,0),L49-M49)),1),0)</x:f>
         <x:v>89</x:v>
       </x:c>
       <x:c r="O49" s="42" t="str">
@@ -5874,7 +5874,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N50" s="40" t="n">
-        <x:f>ROUND(IF(Q50="Não",IF(I50="Não",0,50),MAX(IF(K50&gt;=5,75,0),L50-M50)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q50="Não",IF(I50="Não",0,50),MAX(IF(K50&gt;=5,75,0),L50-M50)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O50" s="42" t="str">
@@ -5943,7 +5943,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N51" s="40" t="n">
-        <x:f>ROUND(IF(Q51="Não",IF(I51="Não",0,50),MAX(IF(K51&gt;=5,75,0),L51-M51)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q51="Não",IF(I51="Não",0,50),MAX(IF(K51&gt;=5,75,0),L51-M51)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O51" s="42" t="str">
@@ -6012,7 +6012,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N52" s="40" t="n">
-        <x:f>ROUND(IF(Q52="Não",IF(I52="Não",0,50),MAX(IF(K52&gt;=5,75,0),L52-M52)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q52="Não",IF(I52="Não",0,50),MAX(IF(K52&gt;=5,75,0),L52-M52)),1),0)</x:f>
         <x:v>79</x:v>
       </x:c>
       <x:c r="O52" s="42" t="str">
@@ -6081,7 +6081,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N53" s="40" t="n">
-        <x:f>ROUND(IF(Q53="Não",IF(I53="Não",0,50),MAX(IF(K53&gt;=5,75,0),L53-M53)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q53="Não",IF(I53="Não",0,50),MAX(IF(K53&gt;=5,75,0),L53-M53)),1),0)</x:f>
         <x:v>79</x:v>
       </x:c>
       <x:c r="O53" s="42" t="str">
@@ -6149,7 +6149,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N54" s="40" t="n">
-        <x:f>ROUND(IF(Q54="Não",IF(I54="Não",0,50),MAX(IF(K54&gt;=5,75,0),L54-M54)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q54="Não",IF(I54="Não",0,50),MAX(IF(K54&gt;=5,75,0),L54-M54)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O54" s="42" t="str">
@@ -6218,7 +6218,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N55" s="40" t="n">
-        <x:f>ROUND(IF(Q55="Não",IF(I55="Não",0,50),MAX(IF(K55&gt;=5,75,0),L55-M55)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q55="Não",IF(I55="Não",0,50),MAX(IF(K55&gt;=5,75,0),L55-M55)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O55" s="42" t="str">
@@ -6287,7 +6287,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N56" s="40" t="n">
-        <x:f>ROUND(IF(Q56="Não",IF(I56="Não",0,50),MAX(IF(K56&gt;=5,75,0),L56-M56)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q56="Não",IF(I56="Não",0,50),MAX(IF(K56&gt;=5,75,0),L56-M56)),1),0)</x:f>
         <x:v>89</x:v>
       </x:c>
       <x:c r="O56" s="42" t="str">
@@ -6356,7 +6356,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N57" s="40" t="n">
-        <x:f>ROUND(IF(Q57="Não",IF(I57="Não",0,50),MAX(IF(K57&gt;=5,75,0),L57-M57)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q57="Não",IF(I57="Não",0,50),MAX(IF(K57&gt;=5,75,0),L57-M57)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O57" s="42" t="str">
@@ -6425,7 +6425,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N58" s="40" t="n">
-        <x:f>ROUND(IF(Q58="Não",IF(I58="Não",0,50),MAX(IF(K58&gt;=5,75,0),L58-M58)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q58="Não",IF(I58="Não",0,50),MAX(IF(K58&gt;=5,75,0),L58-M58)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O58" s="42" t="str">
@@ -6494,7 +6494,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N59" s="40" t="n">
-        <x:f>ROUND(IF(Q59="Não",IF(I59="Não",0,50),MAX(IF(K59&gt;=5,75,0),L59-M59)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q59="Não",IF(I59="Não",0,50),MAX(IF(K59&gt;=5,75,0),L59-M59)),1),0)</x:f>
         <x:v>88</x:v>
       </x:c>
       <x:c r="O59" s="42" t="str">
@@ -6563,7 +6563,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N60" s="40" t="n">
-        <x:f>ROUND(IF(Q60="Não",IF(I60="Não",0,50),MAX(IF(K60&gt;=5,75,0),L60-M60)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q60="Não",IF(I60="Não",0,50),MAX(IF(K60&gt;=5,75,0),L60-M60)),1),0)</x:f>
         <x:v>78</x:v>
       </x:c>
       <x:c r="O60" s="42" t="str">
@@ -6631,7 +6631,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N61" s="40" t="n">
-        <x:f>ROUND(IF(Q61="Não",IF(I61="Não",0,50),MAX(IF(K61&gt;=5,75,0),L61-M61)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q61="Não",IF(I61="Não",0,50),MAX(IF(K61&gt;=5,75,0),L61-M61)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O61" s="42" t="str">
@@ -6700,7 +6700,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N62" s="40" t="n">
-        <x:f>ROUND(IF(Q62="Não",IF(I62="Não",0,50),MAX(IF(K62&gt;=5,75,0),L62-M62)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q62="Não",IF(I62="Não",0,50),MAX(IF(K62&gt;=5,75,0),L62-M62)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O62" s="42" t="str">
@@ -6769,7 +6769,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N63" s="40" t="n">
-        <x:f>ROUND(IF(Q63="Não",IF(I63="Não",0,50),MAX(IF(K63&gt;=5,75,0),L63-M63)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q63="Não",IF(I63="Não",0,50),MAX(IF(K63&gt;=5,75,0),L63-M63)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O63" s="42" t="str">
@@ -6838,7 +6838,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N64" s="40" t="n">
-        <x:f>ROUND(IF(Q64="Não",IF(I64="Não",0,50),MAX(IF(K64&gt;=5,75,0),L64-M64)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q64="Não",IF(I64="Não",0,50),MAX(IF(K64&gt;=5,75,0),L64-M64)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O64" s="42" t="str">
@@ -6907,7 +6907,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N65" s="40" t="n">
-        <x:f>ROUND(IF(Q65="Não",IF(I65="Não",0,50),MAX(IF(K65&gt;=5,75,0),L65-M65)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q65="Não",IF(I65="Não",0,50),MAX(IF(K65&gt;=5,75,0),L65-M65)),1),0)</x:f>
         <x:v>78</x:v>
       </x:c>
       <x:c r="O65" s="42" t="str">
@@ -6975,7 +6975,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N66" s="40" t="n">
-        <x:f>ROUND(IF(Q66="Não",IF(I66="Não",0,50),MAX(IF(K66&gt;=5,75,0),L66-M66)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q66="Não",IF(I66="Não",0,50),MAX(IF(K66&gt;=5,75,0),L66-M66)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O66" s="42" t="str">
@@ -7044,7 +7044,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N67" s="40" t="n">
-        <x:f>ROUND(IF(Q67="Não",IF(I67="Não",0,50),MAX(IF(K67&gt;=5,75,0),L67-M67)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q67="Não",IF(I67="Não",0,50),MAX(IF(K67&gt;=5,75,0),L67-M67)),1),0)</x:f>
         <x:v>80</x:v>
       </x:c>
       <x:c r="O67" s="42" t="str">
@@ -7112,7 +7112,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N68" s="40" t="n">
-        <x:f>ROUND(IF(Q68="Não",IF(I68="Não",0,50),MAX(IF(K68&gt;=5,75,0),L68-M68)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q68="Não",IF(I68="Não",0,50),MAX(IF(K68&gt;=5,75,0),L68-M68)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O68" s="42" t="str">
@@ -7180,7 +7180,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N69" s="40" t="n">
-        <x:f>ROUND(IF(Q69="Não",IF(I69="Não",0,50),MAX(IF(K69&gt;=5,75,0),L69-M69)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q69="Não",IF(I69="Não",0,50),MAX(IF(K69&gt;=5,75,0),L69-M69)),1),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O69" s="42" t="str">
@@ -7248,7 +7248,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N70" s="40" t="n">
-        <x:f>ROUND(IF(Q70="Não",IF(I70="Não",0,50),MAX(IF(K70&gt;=5,75,0),L70-M70)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q70="Não",IF(I70="Não",0,50),MAX(IF(K70&gt;=5,75,0),L70-M70)),1),0)</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="O70" s="42" t="str">
@@ -7317,7 +7317,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N71" s="40" t="n">
-        <x:f>ROUND(IF(Q71="Não",IF(I71="Não",0,50),MAX(IF(K71&gt;=5,75,0),L71-M71)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q71="Não",IF(I71="Não",0,50),MAX(IF(K71&gt;=5,75,0),L71-M71)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O71" s="42" t="str">
@@ -7386,7 +7386,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N72" s="40" t="n">
-        <x:f>ROUND(IF(Q72="Não",IF(I72="Não",0,50),MAX(IF(K72&gt;=5,75,0),L72-M72)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q72="Não",IF(I72="Não",0,50),MAX(IF(K72&gt;=5,75,0),L72-M72)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O72" s="42" t="str">
@@ -7455,7 +7455,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N73" s="40" t="n">
-        <x:f>ROUND(IF(Q73="Não",IF(I73="Não",0,50),MAX(IF(K73&gt;=5,75,0),L73-M73)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q73="Não",IF(I73="Não",0,50),MAX(IF(K73&gt;=5,75,0),L73-M73)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O73" s="42" t="str">
@@ -7524,7 +7524,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N74" s="40" t="n">
-        <x:f>ROUND(IF(Q74="Não",IF(I74="Não",0,50),MAX(IF(K74&gt;=5,75,0),L74-M74)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q74="Não",IF(I74="Não",0,50),MAX(IF(K74&gt;=5,75,0),L74-M74)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O74" s="42" t="str">
@@ -7592,7 +7592,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N75" s="40" t="n">
-        <x:f>ROUND(IF(Q75="Não",IF(I75="Não",0,50),MAX(IF(K75&gt;=5,75,0),L75-M75)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q75="Não",IF(I75="Não",0,50),MAX(IF(K75&gt;=5,75,0),L75-M75)),1),0)</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="O75" s="42" t="str">
@@ -7660,7 +7660,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N76" s="40" t="n">
-        <x:f>ROUND(IF(Q76="Não",IF(I76="Não",0,50),MAX(IF(K76&gt;=5,75,0),L76-M76)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q76="Não",IF(I76="Não",0,50),MAX(IF(K76&gt;=5,75,0),L76-M76)),1),0)</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="O76" s="42" t="str">
@@ -7729,7 +7729,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N77" s="40" t="n">
-        <x:f>ROUND(IF(Q77="Não",IF(I77="Não",0,50),MAX(IF(K77&gt;=5,75,0),L77-M77)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q77="Não",IF(I77="Não",0,50),MAX(IF(K77&gt;=5,75,0),L77-M77)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O77" s="42" t="str">
@@ -7798,7 +7798,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N78" s="40" t="n">
-        <x:f>ROUND(IF(Q78="Não",IF(I78="Não",0,50),MAX(IF(K78&gt;=5,75,0),L78-M78)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q78="Não",IF(I78="Não",0,50),MAX(IF(K78&gt;=5,75,0),L78-M78)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O78" s="42" t="str">
@@ -7867,7 +7867,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N79" s="40" t="n">
-        <x:f>ROUND(IF(Q79="Não",IF(I79="Não",0,50),MAX(IF(K79&gt;=5,75,0),L79-M79)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q79="Não",IF(I79="Não",0,50),MAX(IF(K79&gt;=5,75,0),L79-M79)),1),0)</x:f>
         <x:v>78</x:v>
       </x:c>
       <x:c r="O79" s="42" t="str">
@@ -7936,7 +7936,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N80" s="40" t="n">
-        <x:f>ROUND(IF(Q80="Não",IF(I80="Não",0,50),MAX(IF(K80&gt;=5,75,0),L80-M80)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q80="Não",IF(I80="Não",0,50),MAX(IF(K80&gt;=5,75,0),L80-M80)),1),0)</x:f>
         <x:v>89</x:v>
       </x:c>
       <x:c r="O80" s="42" t="str">
@@ -8005,7 +8005,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N81" s="40" t="n">
-        <x:f>ROUND(IF(Q81="Não",IF(I81="Não",0,50),MAX(IF(K81&gt;=5,75,0),L81-M81)),0)</x:f>
+        <x:f>ROUND(ROUND(IF(Q81="Não",IF(I81="Não",0,50),MAX(IF(K81&gt;=5,75,0),L81-M81)),1),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O81" s="42" t="str">
@@ -8062,7 +8062,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R883d65eae33e41c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref415d026e614aea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8252,7 +8252,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e1fc927379147a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ff07c7695234b03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8472,7 +8472,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1606c90925714fd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c560051a84a42a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>